<commit_message>
Add solution: 0007 - C.
</commit_message>
<xml_diff>
--- a/summary.xlsx
+++ b/summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\EternalSH\GitHub\leetcode\leetcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09E3A196-8B9D-4314-BFEA-2603FCB2EC23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DE4C747-70DC-4A11-A033-60679DA0622D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2480" yWindow="2480" windowWidth="38400" windowHeight="15410" xr2:uid="{4A84287D-0BEF-40C6-AE57-6915C5D67076}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="10">
   <si>
     <t>Problem</t>
   </si>
@@ -544,6 +544,9 @@
       <c r="A8">
         <v>7</v>
       </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
       <c r="C8" t="s">
         <v>4</v>
       </c>

</xml_diff>